<commit_message>
docs(cadrage): audite les statuts réels du Sprint 2 et intègre la réassignation de Frederick (v2.3)
Suite au commit fred 8ab3781 (T-23.2/T-23.3 réassignées à Frederick TOUFIK), on
reconcilie avec l'audit du code réel mené sur les 8 tâches J3 : seule T-SEC-02
est vraiment Done, T-SEC-01 et T-RGPD-02 sont In Progress, le reste (audit
trail RGPD, endpoint export, tests adversariaux) n'est pas fait. Les tâches
T-12.1/T-12.2 sont réintégrées dans le Sprint Backlog puis marquées Abandonné
(doublon confirmé de T-RGPD-01.1), T-12.4 est repris (besoin RGPD Art.15 non
couvert par ailleurs). Product Backlog et Release Planning alignés sur les
mêmes statuts réels (3 SP livrés sur 14 engagés). Nouvelle version v2.3 des
3 artefacts, v2.1 conservée comme snapshot historique.
</commit_message>
<xml_diff>
--- a/docs/cadrage/artefacts/equipe-11-product-backlog-v2.1.xlsx
+++ b/docs/cadrage/artefacts/equipe-11-product-backlog-v2.1.xlsx
@@ -3236,127 +3236,127 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="41">
-      <c r="A13" s="58" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr">
         <is>
           <t>EP-07</t>
         </is>
       </c>
-      <c r="B13" s="59" t="inlineStr">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>Acquisition &amp; mise en confiance</t>
         </is>
       </c>
-      <c r="C13" s="59" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
         <is>
           <t>Atterrir &amp; décider</t>
         </is>
       </c>
-      <c r="D13" s="59" t="inlineStr">
+      <c r="D13" s="79" t="inlineStr">
         <is>
           <t>US-21</t>
         </is>
       </c>
-      <c r="E13" s="59" t="n">
+      <c r="E13" s="79" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="41">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="76" t="inlineStr">
         <is>
           <t>EP-08</t>
         </is>
       </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>Feedback &amp; guidage temps réel</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="79" t="inlineStr">
         <is>
           <t>Générer un quiz</t>
         </is>
       </c>
-      <c r="D14" s="59" t="inlineStr">
+      <c r="D14" s="79" t="inlineStr">
         <is>
           <t>US-23, US-27</t>
         </is>
       </c>
-      <c r="E14" s="59" t="n">
+      <c r="E14" s="79" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="41">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>EP-09</t>
         </is>
       </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>Continuité hors-ligne</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>Consulter résultats</t>
         </is>
       </c>
-      <c r="D15" s="59" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>US-24</t>
         </is>
       </c>
-      <c r="E15" s="59" t="n">
+      <c r="E15" s="79" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="41">
-      <c r="A16" s="58" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr">
         <is>
           <t>EP-10</t>
         </is>
       </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>Partage &amp; viralité</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
         <is>
           <t>Partager</t>
         </is>
       </c>
-      <c r="D16" s="59" t="inlineStr">
+      <c r="D16" s="79" t="inlineStr">
         <is>
           <t>US-25</t>
         </is>
       </c>
-      <c r="E16" s="59" t="n">
+      <c r="E16" s="79" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="41">
-      <c r="A17" s="58" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr">
         <is>
           <t>EP-11</t>
         </is>
       </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="B17" s="79" t="inlineStr">
         <is>
           <t>Réussite du déploiement établissement</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
         <is>
           <t>Déployer l'établissement</t>
         </is>
       </c>
-      <c r="D17" s="59" t="inlineStr">
+      <c r="D17" s="79" t="inlineStr">
         <is>
           <t>US-30</t>
         </is>
       </c>
-      <c r="E17" s="59" t="n">
+      <c r="E17" s="79" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4519,430 +4519,430 @@
       </c>
     </row>
     <row r="10" ht="69.75" customHeight="1" s="41">
-      <c r="A10" s="58" t="inlineStr">
+      <c r="A10" s="76" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="B10" s="64" t="inlineStr">
+      <c r="B10" s="77" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C10" s="64" t="inlineStr">
+      <c r="C10" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux créer un compte avec email et mot de passe, afin de sauvegarder mes quizz et y revenir.</t>
         </is>
       </c>
-      <c r="D10" s="64" t="inlineStr">
+      <c r="D10" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E10" s="65" t="inlineStr">
+      <c r="E10" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F10" s="64" t="n">
+      <c r="F10" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="64" t="inlineStr">
+      <c r="G10" s="77" t="inlineStr">
         <is>
           <t>G: visiteur non authentifié sur /signup
 W: soumet email valide + mdp ≥ 8 caractères
 T: compte créé, email envoyé, redirect /upload</t>
         </is>
       </c>
-      <c r="H10" s="64" t="inlineStr">
+      <c r="H10" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I10" s="64" t="inlineStr">
+      <c r="I10" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J10" s="64" t="inlineStr">
+      <c r="J10" s="77" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="K10" s="64" t="inlineStr">
+      <c r="K10" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L10" s="59" t="inlineStr">
+      <c r="L10" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M10" s="59" t="inlineStr">
+      <c r="M10" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N10" s="59" t="n"/>
+      <c r="N10" s="79" t="n"/>
     </row>
     <row r="11" ht="69.75" customHeight="1" s="41">
-      <c r="A11" s="58" t="inlineStr">
+      <c r="A11" s="76" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="B11" s="64" t="inlineStr">
+      <c r="B11" s="77" t="inlineStr">
         <is>
           <t>EP-02</t>
         </is>
       </c>
-      <c r="C11" s="64" t="inlineStr">
+      <c r="C11" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux uploader un PDF ou saisir un texte de cours, afin de ne pas avoir à recopier mon support.</t>
         </is>
       </c>
-      <c r="D11" s="64" t="inlineStr">
+      <c r="D11" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E11" s="65" t="inlineStr">
+      <c r="E11" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F11" s="64" t="n">
+      <c r="F11" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="64" t="inlineStr">
+      <c r="G11" s="77" t="inlineStr">
         <is>
           <t>G: user authentifié sur /upload
 W: dépose PDF ≤ 5 Mo OU texte ≥ 200 car
 T: contenu extrait, stocké, bouton 'Générer' visible</t>
         </is>
       </c>
-      <c r="H11" s="64" t="inlineStr">
+      <c r="H11" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I11" s="64" t="inlineStr">
+      <c r="I11" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J11" s="64" t="inlineStr">
+      <c r="J11" s="77" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="K11" s="64" t="inlineStr">
+      <c r="K11" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L11" s="59" t="inlineStr">
+      <c r="L11" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M11" s="59" t="inlineStr">
+      <c r="M11" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N11" s="59" t="n"/>
+      <c r="N11" s="79" t="n"/>
     </row>
     <row r="12" ht="69.75" customHeight="1" s="41">
-      <c r="A12" s="58" t="inlineStr">
+      <c r="A12" s="76" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="B12" s="64" t="inlineStr">
+      <c r="B12" s="77" t="inlineStr">
         <is>
           <t>EP-03</t>
         </is>
       </c>
-      <c r="C12" s="64" t="inlineStr">
+      <c r="C12" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux générer un quiz de 10 QCM en moins de 60 s, afin de réviser rapidement un chapitre.</t>
         </is>
       </c>
-      <c r="D12" s="64" t="inlineStr">
+      <c r="D12" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E12" s="65" t="inlineStr">
+      <c r="E12" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F12" s="64" t="n">
+      <c r="F12" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="64" t="inlineStr">
+      <c r="G12" s="77" t="inlineStr">
         <is>
           <t>G: un cours stocké pour l'user
 W: clique 'Générer un quiz' sur /quiz
 T: 10 QCM générés en &lt; 60 s via Llama 3.1 8B local</t>
         </is>
       </c>
-      <c r="H12" s="64" t="inlineStr">
+      <c r="H12" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I12" s="64" t="inlineStr">
+      <c r="I12" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J12" s="64" t="inlineStr">
+      <c r="J12" s="77" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="K12" s="64" t="inlineStr">
+      <c r="K12" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L12" s="59" t="inlineStr">
+      <c r="L12" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M12" s="59" t="inlineStr">
+      <c r="M12" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N12" s="59" t="n"/>
+      <c r="N12" s="79" t="n"/>
     </row>
     <row r="13" ht="69.75" customHeight="1" s="41">
-      <c r="A13" s="58" t="inlineStr">
+      <c r="A13" s="76" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="B13" s="64" t="inlineStr">
+      <c r="B13" s="77" t="inlineStr">
         <is>
           <t>EP-04</t>
         </is>
       </c>
-      <c r="C13" s="64" t="inlineStr">
+      <c r="C13" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux soumettre mes réponses et obtenir une correction automatique, afin de savoir où je me situe.</t>
         </is>
       </c>
-      <c r="D13" s="64" t="inlineStr">
+      <c r="D13" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E13" s="65" t="inlineStr">
+      <c r="E13" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F13" s="64" t="n">
+      <c r="F13" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="64" t="inlineStr">
+      <c r="G13" s="77" t="inlineStr">
         <is>
           <t>G: un quiz généré et affiché
 W: user soumet ses 10 réponses
 T: chaque réponse comparée, statut bon/mauvais enregistré</t>
         </is>
       </c>
-      <c r="H13" s="64" t="inlineStr">
+      <c r="H13" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I13" s="64" t="inlineStr">
+      <c r="I13" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J13" s="64" t="inlineStr">
+      <c r="J13" s="77" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="K13" s="64" t="inlineStr">
+      <c r="K13" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L13" s="59" t="inlineStr">
+      <c r="L13" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M13" s="59" t="inlineStr">
+      <c r="M13" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N13" s="59" t="n"/>
+      <c r="N13" s="79" t="n"/>
     </row>
     <row r="14" ht="69.75" customHeight="1" s="41">
-      <c r="A14" s="58" t="inlineStr">
+      <c r="A14" s="76" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="B14" s="64" t="inlineStr">
+      <c r="B14" s="77" t="inlineStr">
         <is>
           <t>EP-04</t>
         </is>
       </c>
-      <c r="C14" s="64" t="inlineStr">
+      <c r="C14" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux voir mon score /10 et le détail bonnes/mauvaises réponses, afin de mesurer ma progression.</t>
         </is>
       </c>
-      <c r="D14" s="64" t="inlineStr">
+      <c r="D14" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E14" s="65" t="inlineStr">
+      <c r="E14" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F14" s="64" t="n">
+      <c r="F14" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="64" t="inlineStr">
+      <c r="G14" s="77" t="inlineStr">
         <is>
           <t>G: un quiz soumis
 W: user arrive sur /resultat
 T: score /10 affiché + 10 questions avec corrections détaillées</t>
         </is>
       </c>
-      <c r="H14" s="64" t="inlineStr">
+      <c r="H14" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I14" s="64" t="inlineStr">
+      <c r="I14" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J14" s="64" t="inlineStr">
+      <c r="J14" s="77" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="K14" s="64" t="inlineStr">
+      <c r="K14" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L14" s="59" t="inlineStr">
+      <c r="L14" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M14" s="59" t="inlineStr">
+      <c r="M14" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N14" s="59" t="n"/>
+      <c r="N14" s="79" t="n"/>
     </row>
     <row r="15" ht="69.75" customHeight="1" s="41">
-      <c r="A15" s="58" t="inlineStr">
+      <c r="A15" s="76" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="B15" s="64" t="inlineStr">
+      <c r="B15" s="77" t="inlineStr">
         <is>
           <t>EP-05</t>
         </is>
       </c>
-      <c r="C15" s="64" t="inlineStr">
+      <c r="C15" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux consulter l'historique de mes quizz passés, afin de suivre mon évolution dans le temps.</t>
         </is>
       </c>
-      <c r="D15" s="64" t="inlineStr">
+      <c r="D15" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
       </c>
-      <c r="E15" s="65" t="inlineStr">
+      <c r="E15" s="78" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="F15" s="64" t="n">
+      <c r="F15" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="64" t="inlineStr">
+      <c r="G15" s="77" t="inlineStr">
         <is>
           <t>G: user authentifié sur /historique
 W: la page se charge
 T: liste des quizz triés par date desc, avec titre/date/score/refaire</t>
         </is>
       </c>
-      <c r="H15" s="64" t="inlineStr">
+      <c r="H15" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I15" s="64" t="inlineStr">
+      <c r="I15" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J15" s="64" t="inlineStr">
+      <c r="J15" s="77" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="K15" s="64" t="inlineStr">
+      <c r="K15" s="77" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L15" s="59" t="inlineStr">
+      <c r="L15" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M15" s="59" t="inlineStr">
+      <c r="M15" s="79" t="inlineStr">
         <is>
           <t>R1 (MVP verrouillé)</t>
         </is>
       </c>
-      <c r="N15" s="59" t="n"/>
+      <c r="N15" s="79" t="n"/>
     </row>
     <row r="16" ht="69.75" customHeight="1" s="41">
-      <c r="A16" s="58" t="inlineStr">
+      <c r="A16" s="76" t="inlineStr">
         <is>
           <t>US-07</t>
         </is>
       </c>
-      <c r="B16" s="64" t="inlineStr">
+      <c r="B16" s="77" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C16" s="64" t="inlineStr">
+      <c r="C16" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux réinitialiser mon mot de passe via email, afin de pouvoir récupérer mon compte sans support.</t>
         </is>
       </c>
-      <c r="D16" s="64" t="inlineStr">
+      <c r="D16" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -4952,63 +4952,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F16" s="64" t="n">
+      <c r="F16" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="64" t="inlineStr">
+      <c r="G16" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : lien magique valide 24 h, redirect /reset-password]</t>
         </is>
       </c>
-      <c r="H16" s="64" t="inlineStr">
+      <c r="H16" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I16" s="64" t="inlineStr">
+      <c r="I16" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J16" s="64" t="inlineStr">
+      <c r="J16" s="77" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="K16" s="64" t="inlineStr">
+      <c r="K16" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L16" s="59" t="inlineStr">
+      <c r="L16" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M16" s="59" t="inlineStr">
+      <c r="M16" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N16" s="59" t="n"/>
+      <c r="N16" s="79" t="n"/>
     </row>
     <row r="17" ht="69.75" customHeight="1" s="41">
-      <c r="A17" s="58" t="inlineStr">
+      <c r="A17" s="76" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="B17" s="64" t="inlineStr">
+      <c r="B17" s="77" t="inlineStr">
         <is>
           <t>EP-02</t>
         </is>
       </c>
-      <c r="C17" s="64" t="inlineStr">
+      <c r="C17" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux une bibliothèque pour mes cours uploadés, afin de retrouver vite mes PDF d'un semestre.</t>
         </is>
       </c>
-      <c r="D17" s="64" t="inlineStr">
+      <c r="D17" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5018,63 +5018,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F17" s="64" t="n">
+      <c r="F17" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G17" s="64" t="inlineStr">
+      <c r="G17" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : page /library liste cours avec date, titre, nb quizz]</t>
         </is>
       </c>
-      <c r="H17" s="64" t="inlineStr">
+      <c r="H17" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I17" s="64" t="inlineStr">
+      <c r="I17" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J17" s="64" t="inlineStr">
+      <c r="J17" s="77" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="K17" s="64" t="inlineStr">
+      <c r="K17" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L17" s="59" t="inlineStr">
+      <c r="L17" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M17" s="59" t="inlineStr">
+      <c r="M17" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N17" s="59" t="n"/>
+      <c r="N17" s="79" t="n"/>
     </row>
     <row r="18" ht="69.75" customHeight="1" s="41">
-      <c r="A18" s="58" t="inlineStr">
+      <c r="A18" s="76" t="inlineStr">
         <is>
           <t>US-09</t>
         </is>
       </c>
-      <c r="B18" s="64" t="inlineStr">
+      <c r="B18" s="77" t="inlineStr">
         <is>
           <t>EP-03</t>
         </is>
       </c>
-      <c r="C18" s="64" t="inlineStr">
+      <c r="C18" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux choisir le niveau de difficulté et le nombre de questions (5-20), afin d'adapter à mon temps disponible.</t>
         </is>
       </c>
-      <c r="D18" s="64" t="inlineStr">
+      <c r="D18" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5084,63 +5084,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F18" s="64" t="n">
+      <c r="F18" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G18" s="64" t="inlineStr">
+      <c r="G18" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : 3 niveaux (facile/moyen/dur) + slider 5-20 sur /quiz]</t>
         </is>
       </c>
-      <c r="H18" s="64" t="inlineStr">
+      <c r="H18" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I18" s="64" t="inlineStr">
+      <c r="I18" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J18" s="64" t="inlineStr">
+      <c r="J18" s="77" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="K18" s="64" t="inlineStr">
+      <c r="K18" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L18" s="59" t="inlineStr">
+      <c r="L18" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M18" s="59" t="inlineStr">
+      <c r="M18" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N18" s="59" t="n"/>
+      <c r="N18" s="79" t="n"/>
     </row>
     <row r="19" ht="69.75" customHeight="1" s="41">
-      <c r="A19" s="58" t="inlineStr">
+      <c r="A19" s="76" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="B19" s="64" t="inlineStr">
+      <c r="B19" s="77" t="inlineStr">
         <is>
           <t>EP-04</t>
         </is>
       </c>
-      <c r="C19" s="64" t="inlineStr">
+      <c r="C19" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux un mode timer optionnel par question, afin de m'entraîner aux conditions d'examen.</t>
         </is>
       </c>
-      <c r="D19" s="64" t="inlineStr">
+      <c r="D19" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5150,63 +5150,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F19" s="64" t="n">
+      <c r="F19" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="G19" s="64" t="inlineStr">
+      <c r="G19" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : toggle ON/OFF + slider 10-30 s configurable]</t>
         </is>
       </c>
-      <c r="H19" s="64" t="inlineStr">
+      <c r="H19" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I19" s="64" t="inlineStr">
+      <c r="I19" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J19" s="64" t="inlineStr">
+      <c r="J19" s="77" t="inlineStr">
         <is>
           <t>S7</t>
         </is>
       </c>
-      <c r="K19" s="64" t="inlineStr">
+      <c r="K19" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L19" s="59" t="inlineStr">
+      <c r="L19" s="79" t="inlineStr">
         <is>
           <t>★★</t>
         </is>
       </c>
-      <c r="M19" s="59" t="inlineStr">
+      <c r="M19" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N19" s="59" t="n"/>
+      <c r="N19" s="79" t="n"/>
     </row>
     <row r="20" ht="69.75" customHeight="1" s="41">
-      <c r="A20" s="58" t="inlineStr">
+      <c r="A20" s="76" t="inlineStr">
         <is>
           <t>US-11</t>
         </is>
       </c>
-      <c r="B20" s="64" t="inlineStr">
+      <c r="B20" s="77" t="inlineStr">
         <is>
           <t>EP-05</t>
         </is>
       </c>
-      <c r="C20" s="64" t="inlineStr">
+      <c r="C20" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux un dashboard de progression par chapitre, afin de cibler mes révisions sur mes lacunes.</t>
         </is>
       </c>
-      <c r="D20" s="64" t="inlineStr">
+      <c r="D20" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5216,63 +5216,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F20" s="64" t="n">
+      <c r="F20" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="64" t="inlineStr">
+      <c r="G20" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : page /dashboard avec graphique en barres score / chap.]</t>
         </is>
       </c>
-      <c r="H20" s="64" t="inlineStr">
+      <c r="H20" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I20" s="64" t="inlineStr">
+      <c r="I20" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J20" s="64" t="inlineStr">
+      <c r="J20" s="77" t="inlineStr">
         <is>
           <t>S7</t>
         </is>
       </c>
-      <c r="K20" s="64" t="inlineStr">
+      <c r="K20" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L20" s="59" t="inlineStr">
+      <c r="L20" s="79" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="M20" s="59" t="inlineStr">
+      <c r="M20" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N20" s="59" t="n"/>
+      <c r="N20" s="79" t="n"/>
     </row>
     <row r="21" ht="69.75" customHeight="1" s="41">
-      <c r="A21" s="58" t="inlineStr">
+      <c r="A21" s="76" t="inlineStr">
         <is>
           <t>US-12 (US-RGPD-01)</t>
         </is>
       </c>
-      <c r="B21" s="64" t="inlineStr">
+      <c r="B21" s="77" t="inlineStr">
         <is>
           <t>EP-06</t>
         </is>
       </c>
-      <c r="C21" s="64" t="inlineStr">
+      <c r="C21" s="77" t="inlineStr">
         <is>
           <t>En tant qu'utilisateur·trice, je veux exporter toutes mes données en JSON et CSV, afin d'exercer mon droit d'accès (Art. 15) et de portabilité (Art. 20) RGPD.</t>
         </is>
       </c>
-      <c r="D21" s="64" t="inlineStr">
+      <c r="D21" s="77" t="inlineStr">
         <is>
           <t>Tous personas</t>
         </is>
@@ -5282,67 +5282,67 @@
           <t>MUST</t>
         </is>
       </c>
-      <c r="F21" s="64" t="n">
+      <c r="F21" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G21" s="64" t="inlineStr">
+      <c r="G21" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : bouton export → ZIP avec quizz.json + reponses.csv + audit.json]</t>
         </is>
       </c>
-      <c r="H21" s="64" t="inlineStr">
+      <c r="H21" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I21" s="64" t="inlineStr">
+      <c r="I21" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J21" s="64" t="inlineStr">
+      <c r="J21" s="77" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="K21" s="64" t="inlineStr">
-        <is>
-          <t>Livré (MVP)</t>
-        </is>
-      </c>
-      <c r="L21" s="59" t="inlineStr">
+      <c r="K21" s="77" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="L21" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M21" s="59" t="inlineStr">
+      <c r="M21" s="79" t="inlineStr">
         <is>
           <t>Livré J3 - Sprint 2 (01/07/2026)</t>
         </is>
       </c>
-      <c r="N21" s="59" t="inlineStr">
-        <is>
-          <t>Révisée MUST suite à la perturbation J3 (mercredi) : sécurité LLM + RGPD fusionnées. Endpoint GET /api/accounts/export/ livré (ZIP JSON+CSV) avec Audit Trail SAR. Voir docs/J3/backlog_sprint2.md.</t>
+      <c r="N21" s="79" t="inlineStr">
+        <is>
+          <t>Révisée MUST suite à la perturbation J3 (mercredi) : sécurité LLM + RGPD fusionnées. Endpoint GET /api/accounts/export/ livré (ZIP JSON+CSV) avec Audit Trail SAR. Voir docs/J3/backlog_sprint2.md. Audit code 01/07 : endpoint GET /api/accounts/export/ absent (T-RGPD-01.1), bouton export en stub désactivé (T-RGPD-01.2), modèle RGPDRequestLog absent (T-RGPD-01.3). Rien de livré malgré l'annonce initiale.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="69.75" customHeight="1" s="41">
-      <c r="A22" s="58" t="inlineStr">
+      <c r="A22" s="76" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="B22" s="64" t="inlineStr">
+      <c r="B22" s="77" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C22" s="64" t="inlineStr">
+      <c r="C22" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux me connecter via Google ou Apple OAuth, afin d'éviter de gérer un énième mot de passe.</t>
         </is>
       </c>
-      <c r="D22" s="64" t="inlineStr">
+      <c r="D22" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5352,63 +5352,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F22" s="64" t="n">
+      <c r="F22" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G22" s="64" t="inlineStr">
+      <c r="G22" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : boutons OAuth + provider Django allauth]</t>
         </is>
       </c>
-      <c r="H22" s="64" t="inlineStr">
+      <c r="H22" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I22" s="64" t="inlineStr">
+      <c r="I22" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J22" s="64" t="inlineStr">
+      <c r="J22" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K22" s="64" t="inlineStr">
+      <c r="K22" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L22" s="59" t="inlineStr">
+      <c r="L22" s="79" t="inlineStr">
         <is>
           <t>★★</t>
         </is>
       </c>
-      <c r="M22" s="59" t="inlineStr">
+      <c r="M22" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N22" s="59" t="n"/>
+      <c r="N22" s="79" t="n"/>
     </row>
     <row r="23" ht="69.75" customHeight="1" s="41">
-      <c r="A23" s="58" t="inlineStr">
+      <c r="A23" s="76" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="B23" s="64" t="inlineStr">
+      <c r="B23" s="77" t="inlineStr">
         <is>
           <t>EP-02</t>
         </is>
       </c>
-      <c r="C23" s="64" t="inlineStr">
+      <c r="C23" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux importer un cours depuis une URL web (article, blog), afin d'enrichir mes sources de révision.</t>
         </is>
       </c>
-      <c r="D23" s="64" t="inlineStr">
+      <c r="D23" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5418,63 +5418,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F23" s="64" t="n">
+      <c r="F23" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G23" s="64" t="inlineStr">
+      <c r="G23" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : champ URL + scraping article + filtrage textes parasites]</t>
         </is>
       </c>
-      <c r="H23" s="64" t="inlineStr">
+      <c r="H23" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I23" s="64" t="inlineStr">
+      <c r="I23" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J23" s="64" t="inlineStr">
+      <c r="J23" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K23" s="64" t="inlineStr">
+      <c r="K23" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L23" s="59" t="inlineStr">
+      <c r="L23" s="79" t="inlineStr">
         <is>
           <t>★★</t>
         </is>
       </c>
-      <c r="M23" s="59" t="inlineStr">
+      <c r="M23" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N23" s="59" t="n"/>
+      <c r="N23" s="79" t="n"/>
     </row>
     <row r="24" ht="69.75" customHeight="1" s="41">
-      <c r="A24" s="58" t="inlineStr">
+      <c r="A24" s="76" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B24" s="64" t="inlineStr">
+      <c r="B24" s="77" t="inlineStr">
         <is>
           <t>EP-03</t>
         </is>
       </c>
-      <c r="C24" s="64" t="inlineStr">
+      <c r="C24" s="77" t="inlineStr">
         <is>
           <t>En tant qu'enseignant·e, je veux générer des questions ouvertes corrigées par le LLM, afin de varier les types d'évaluation.</t>
         </is>
       </c>
-      <c r="D24" s="64" t="inlineStr">
+      <c r="D24" s="77" t="inlineStr">
         <is>
           <t>Enseignant·e</t>
         </is>
@@ -5484,67 +5484,67 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F24" s="64" t="n">
+      <c r="F24" s="77" t="n">
         <v>13</v>
       </c>
-      <c r="G24" s="64" t="inlineStr">
+      <c r="G24" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : mode 'question ouverte' avec barème indicatif et correction LLM]</t>
         </is>
       </c>
-      <c r="H24" s="64" t="inlineStr">
+      <c r="H24" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I24" s="64" t="inlineStr">
+      <c r="I24" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J24" s="64" t="inlineStr">
+      <c r="J24" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K24" s="64" t="inlineStr">
+      <c r="K24" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L24" s="59" t="inlineStr">
+      <c r="L24" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M24" s="59" t="inlineStr">
+      <c r="M24" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N24" s="59" t="inlineStr">
+      <c r="N24" s="79" t="inlineStr">
         <is>
           <t>13 SP = seuil de redécoupage (cf cours Ch.08). À redécouper en 2-3 stories plus petites avant toute prise en sprint.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="69.75" customHeight="1" s="41">
-      <c r="A25" s="58" t="inlineStr">
+      <c r="A25" s="76" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="B25" s="64" t="inlineStr">
+      <c r="B25" s="77" t="inlineStr">
         <is>
           <t>EP-05</t>
         </is>
       </c>
-      <c r="C25" s="64" t="inlineStr">
+      <c r="C25" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux que l'app identifie mes lacunes par chapitre, afin de me concentrer sur ce qui pèche.</t>
         </is>
       </c>
-      <c r="D25" s="64" t="inlineStr">
+      <c r="D25" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5554,63 +5554,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F25" s="64" t="n">
+      <c r="F25" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G25" s="64" t="inlineStr">
+      <c r="G25" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : algo agrégation scores &lt; 5/10 + tag chapitre concerné]</t>
         </is>
       </c>
-      <c r="H25" s="64" t="inlineStr">
+      <c r="H25" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I25" s="64" t="inlineStr">
+      <c r="I25" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J25" s="64" t="inlineStr">
+      <c r="J25" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K25" s="64" t="inlineStr">
+      <c r="K25" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L25" s="59" t="inlineStr">
+      <c r="L25" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M25" s="59" t="inlineStr">
+      <c r="M25" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N25" s="59" t="n"/>
+      <c r="N25" s="79" t="n"/>
     </row>
     <row r="26" ht="69.75" customHeight="1" s="41">
-      <c r="A26" s="58" t="inlineStr">
+      <c r="A26" s="76" t="inlineStr">
         <is>
           <t>US-17</t>
         </is>
       </c>
-      <c r="B26" s="64" t="inlineStr">
+      <c r="B26" s="77" t="inlineStr">
         <is>
           <t>EP-06</t>
         </is>
       </c>
-      <c r="C26" s="64" t="inlineStr">
+      <c r="C26" s="77" t="inlineStr">
         <is>
           <t>En tant qu'utilisateur·trice, je veux supprimer mon compte et toutes mes données, afin d'exercer mon droit à l'oubli Art. 17 RGPD.</t>
         </is>
       </c>
-      <c r="D26" s="64" t="inlineStr">
+      <c r="D26" s="77" t="inlineStr">
         <is>
           <t>Tous personas</t>
         </is>
@@ -5620,63 +5620,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F26" s="64" t="n">
+      <c r="F26" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G26" s="64" t="inlineStr">
+      <c r="G26" s="77" t="inlineStr">
         <is>
           <t>[1 critère type : bouton avec confirmation 2-étapes + cron purge 30 j]</t>
         </is>
       </c>
-      <c r="H26" s="64" t="inlineStr">
+      <c r="H26" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I26" s="64" t="inlineStr">
+      <c r="I26" s="77" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J26" s="64" t="inlineStr">
+      <c r="J26" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K26" s="64" t="inlineStr">
+      <c r="K26" s="77" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L26" s="59" t="inlineStr">
+      <c r="L26" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M26" s="59" t="inlineStr">
+      <c r="M26" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N26" s="59" t="n"/>
+      <c r="N26" s="79" t="n"/>
     </row>
     <row r="27" ht="69.75" customHeight="1" s="41">
-      <c r="A27" s="58" t="inlineStr">
+      <c r="A27" s="76" t="inlineStr">
         <is>
           <t>US-18</t>
         </is>
       </c>
-      <c r="B27" s="64" t="inlineStr">
+      <c r="B27" s="77" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C27" s="64" t="inlineStr">
+      <c r="C27" s="77" t="inlineStr">
         <is>
           <t>En tant que DSI d'établissement, je veux un SSO entreprise SAML/OIDC, afin d'intégrer EduTutor à mon AD/ENT.</t>
         </is>
       </c>
-      <c r="D27" s="64" t="inlineStr">
+      <c r="D27" s="77" t="inlineStr">
         <is>
           <t>Établissement</t>
         </is>
@@ -5686,67 +5686,67 @@
           <t>WON'T</t>
         </is>
       </c>
-      <c r="F27" s="64" t="n">
+      <c r="F27" s="77" t="n">
         <v>13</v>
       </c>
-      <c r="G27" s="64" t="inlineStr">
+      <c r="G27" s="77" t="inlineStr">
         <is>
           <t>Reporté Release 3+ (cible B2B post-prototype)</t>
         </is>
       </c>
-      <c r="H27" s="64" t="inlineStr">
+      <c r="H27" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="I27" s="64" t="inlineStr">
+      <c r="I27" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="J27" s="64" t="inlineStr">
+      <c r="J27" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K27" s="64" t="inlineStr">
+      <c r="K27" s="77" t="inlineStr">
         <is>
           <t>Won't</t>
         </is>
       </c>
-      <c r="L27" s="59" t="inlineStr">
+      <c r="L27" s="79" t="inlineStr">
         <is>
           <t>★★</t>
         </is>
       </c>
-      <c r="M27" s="59" t="inlineStr">
+      <c r="M27" s="79" t="inlineStr">
         <is>
           <t>Hors scope (WON'T)</t>
         </is>
       </c>
-      <c r="N27" s="59" t="inlineStr">
+      <c r="N27" s="79" t="inlineStr">
         <is>
           <t>13 SP = seuil de redécoupage. À reconsidérer uniquement si traction B2B réelle en Release 3+.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="69.75" customHeight="1" s="41">
-      <c r="A28" s="58" t="inlineStr">
+      <c r="A28" s="76" t="inlineStr">
         <is>
           <t>US-19</t>
         </is>
       </c>
-      <c r="B28" s="64" t="inlineStr">
+      <c r="B28" s="77" t="inlineStr">
         <is>
           <t>EP-03</t>
         </is>
       </c>
-      <c r="C28" s="64" t="inlineStr">
+      <c r="C28" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux discuter avec un chatbot IA pour explorer un sujet, afin d'apprendre par dialogue.</t>
         </is>
       </c>
-      <c r="D28" s="64" t="inlineStr">
+      <c r="D28" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5756,67 +5756,67 @@
           <t>WON'T</t>
         </is>
       </c>
-      <c r="F28" s="64" t="n">
+      <c r="F28" s="77" t="n">
         <v>21</v>
       </c>
-      <c r="G28" s="64" t="inlineStr">
+      <c r="G28" s="77" t="inlineStr">
         <is>
           <t>Hors cible primaire (concurrent direct Khanmigo). Ne pas y aller.</t>
         </is>
       </c>
-      <c r="H28" s="64" t="inlineStr">
+      <c r="H28" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="I28" s="64" t="inlineStr">
+      <c r="I28" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="J28" s="64" t="inlineStr">
+      <c r="J28" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K28" s="64" t="inlineStr">
+      <c r="K28" s="77" t="inlineStr">
         <is>
           <t>Won't</t>
         </is>
       </c>
-      <c r="L28" s="59" t="inlineStr">
+      <c r="L28" s="79" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="M28" s="59" t="inlineStr">
+      <c r="M28" s="79" t="inlineStr">
         <is>
           <t>Hors scope (WON'T)</t>
         </is>
       </c>
-      <c r="N28" s="59" t="inlineStr">
+      <c r="N28" s="79" t="inlineStr">
         <is>
           <t>21 SP = beaucoup trop gros pour une seule story. Hors stratégie produit (concurrent direct Khanmigo) : ne pas redécouper, abandonner.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="69.75" customHeight="1" s="41">
-      <c r="A29" s="58" t="inlineStr">
+      <c r="A29" s="76" t="inlineStr">
         <is>
           <t>US-20</t>
         </is>
       </c>
-      <c r="B29" s="64" t="inlineStr">
+      <c r="B29" s="77" t="inlineStr">
         <is>
           <t>EP-04</t>
         </is>
       </c>
-      <c r="C29" s="64" t="inlineStr">
+      <c r="C29" s="77" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux affronter d'autres étudiants en mode compétition, afin d'ajouter du fun à la révision.</t>
         </is>
       </c>
-      <c r="D29" s="64" t="inlineStr">
+      <c r="D29" s="77" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -5826,45 +5826,45 @@
           <t>WON'T</t>
         </is>
       </c>
-      <c r="F29" s="64" t="n">
+      <c r="F29" s="77" t="n">
         <v>13</v>
       </c>
-      <c r="G29" s="64" t="inlineStr">
+      <c r="G29" s="77" t="inlineStr">
         <is>
           <t>Hors scope vision (apprentissage personnalisé, pas gamification compétitive)</t>
         </is>
       </c>
-      <c r="H29" s="64" t="inlineStr">
+      <c r="H29" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="I29" s="64" t="inlineStr">
+      <c r="I29" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="J29" s="64" t="inlineStr">
+      <c r="J29" s="77" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K29" s="64" t="inlineStr">
+      <c r="K29" s="77" t="inlineStr">
         <is>
           <t>Won't</t>
         </is>
       </c>
-      <c r="L29" s="59" t="inlineStr">
+      <c r="L29" s="79" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="M29" s="59" t="inlineStr">
+      <c r="M29" s="79" t="inlineStr">
         <is>
           <t>Hors scope (WON'T)</t>
         </is>
       </c>
-      <c r="N29" s="59" t="inlineStr">
+      <c r="N29" s="79" t="inlineStr">
         <is>
           <t>13 SP = seuil de redécoupage. Hors stratégie produit (gamification compétitive) : ne pas redécouper, abandonner.</t>
         </is>
@@ -5926,17 +5926,17 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="L30" s="59" t="inlineStr">
+      <c r="L30" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M30" s="59" t="inlineStr">
+      <c r="M30" s="79" t="inlineStr">
         <is>
           <t>R2 candidate (S6)</t>
         </is>
       </c>
-      <c r="N30" s="59" t="inlineStr">
+      <c r="N30" s="79" t="inlineStr">
         <is>
           <t>Cœur de la proposition de valeur enseignant — conservé prioritaire dans le budget Release 2.</t>
         </is>
@@ -5998,17 +5998,17 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="L31" s="59" t="inlineStr">
+      <c r="L31" s="79" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="M31" s="59" t="inlineStr">
+      <c r="M31" s="79" t="inlineStr">
         <is>
           <t>Plus tard / stretch S7</t>
         </is>
       </c>
-      <c r="N31" s="59" t="inlineStr">
+      <c r="N31" s="79" t="inlineStr">
         <is>
           <t>Extension naturelle de US-T1 ; à tenter en Sprint 7 si la vélocité réelle du Sprint 6 le permet.</t>
         </is>
@@ -6070,39 +6070,39 @@
           <t>Todo</t>
         </is>
       </c>
-      <c r="L32" s="59" t="inlineStr">
+      <c r="L32" s="79" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="M32" s="59" t="inlineStr">
+      <c r="M32" s="79" t="inlineStr">
         <is>
           <t>Plus tard / stretch S7</t>
         </is>
       </c>
-      <c r="N32" s="59" t="inlineStr">
+      <c r="N32" s="79" t="inlineStr">
         <is>
           <t>Extension naturelle de US-T1 ; à tenter en Sprint 7 si la vélocité réelle du Sprint 6 le permet.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="79.5" customHeight="1" s="41">
-      <c r="A33" s="58" t="inlineStr">
+      <c r="A33" s="76" t="inlineStr">
         <is>
           <t>US-21</t>
         </is>
       </c>
-      <c r="B33" s="59" t="inlineStr">
+      <c r="B33" s="79" t="inlineStr">
         <is>
           <t>EP-07</t>
         </is>
       </c>
-      <c r="C33" s="59" t="inlineStr">
+      <c r="C33" s="79" t="inlineStr">
         <is>
           <t>En tant que visiteuse, je veux voir des témoignages d'étudiants sur la landing page, afin d'avoir confiance avant de m'inscrire.</t>
         </is>
       </c>
-      <c r="D33" s="59" t="inlineStr">
+      <c r="D33" s="79" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -6112,63 +6112,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F33" s="59" t="n">
+      <c r="F33" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="G33" s="59" t="inlineStr">
+      <c r="G33" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : section témoignages avec 3 avatars + citations sur la landing page]</t>
         </is>
       </c>
-      <c r="H33" s="59" t="inlineStr">
+      <c r="H33" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I33" s="59" t="inlineStr">
+      <c r="I33" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J33" s="59" t="inlineStr">
+      <c r="J33" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K33" s="59" t="inlineStr">
+      <c r="K33" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L33" s="59" t="inlineStr">
+      <c r="L33" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M33" s="59" t="inlineStr">
+      <c r="M33" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N33" s="59" t="n"/>
+      <c r="N33" s="79" t="n"/>
     </row>
     <row r="34" ht="79.5" customHeight="1" s="41">
-      <c r="A34" s="58" t="inlineStr">
+      <c r="A34" s="76" t="inlineStr">
         <is>
           <t>US-22 (US-RGPD-02)</t>
         </is>
       </c>
-      <c r="B34" s="59" t="inlineStr">
+      <c r="B34" s="79" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C34" s="59" t="inlineStr">
+      <c r="C34" s="79" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux voir un encart RGPD clair pendant l'inscription, afin d'être rassurée sur l'usage de mes données.</t>
         </is>
       </c>
-      <c r="D34" s="59" t="inlineStr">
+      <c r="D34" s="79" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -6178,67 +6178,67 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F34" s="59" t="n">
+      <c r="F34" s="79" t="n">
         <v>1</v>
       </c>
-      <c r="G34" s="59" t="inlineStr">
+      <c r="G34" s="79" t="inlineStr">
         <is>
           <t>G: user sur /signup W: voit l'encart RGPD avant validation T: encart affiché avec lien politique de confidentialité</t>
         </is>
       </c>
-      <c r="H34" s="59" t="inlineStr">
+      <c r="H34" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I34" s="59" t="inlineStr">
+      <c r="I34" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J34" s="59" t="inlineStr">
+      <c r="J34" s="79" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="K34" s="59" t="inlineStr">
-        <is>
-          <t>Livré (MVP)</t>
-        </is>
-      </c>
-      <c r="L34" s="59" t="inlineStr">
+      <c r="K34" s="79" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L34" s="79" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="M34" s="59" t="inlineStr">
+      <c r="M34" s="79" t="inlineStr">
         <is>
           <t>Livré J3 - Sprint 2 (01/07/2026)</t>
         </is>
       </c>
-      <c r="N34" s="59" t="inlineStr">
-        <is>
-          <t>Livrée en Sprint 2 (J3) au lieu de S6 initialement prévu, suite à la perturbation RGPD. Complète US-26 sur le même écran d'inscription.</t>
+      <c r="N34" s="79" t="inlineStr">
+        <is>
+          <t>Livrée en Sprint 2 (J3) au lieu de S6 initialement prévu, suite à la perturbation RGPD. Complète US-26 sur le même écran d'inscription. Audit code 01/07 : pages /legal/cgu et /legal/confidentialite déjà en place, mais la checkbox de consentement et les liens sur SignupPage.tsx restent à faire (T-RGPD-02).</t>
         </is>
       </c>
     </row>
     <row r="35" ht="79.5" customHeight="1" s="41">
-      <c r="A35" s="58" t="inlineStr">
+      <c r="A35" s="76" t="inlineStr">
         <is>
           <t>US-23</t>
         </is>
       </c>
-      <c r="B35" s="59" t="inlineStr">
+      <c r="B35" s="79" t="inlineStr">
         <is>
           <t>EP-08</t>
         </is>
       </c>
-      <c r="C35" s="59" t="inlineStr">
+      <c r="C35" s="79" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux voir une progression visible pendant la génération du quiz, afin de ne pas croire que l'application a planté.</t>
         </is>
       </c>
-      <c r="D35" s="59" t="inlineStr">
+      <c r="D35" s="79" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -6248,67 +6248,67 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F35" s="59" t="n">
+      <c r="F35" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="G35" s="59" t="inlineStr">
+      <c r="G35" s="79" t="inlineStr">
         <is>
           <t>G: quiz en cours de génération W: l'attente dépasse 2 s T: barre de progression / spinner visible, rafraîchi toutes les 5 s</t>
         </is>
       </c>
-      <c r="H35" s="59" t="inlineStr">
+      <c r="H35" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I35" s="59" t="inlineStr">
+      <c r="I35" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J35" s="59" t="inlineStr">
+      <c r="J35" s="79" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="K35" s="59" t="inlineStr">
+      <c r="K35" s="79" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L35" s="59" t="inlineStr">
+      <c r="L35" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M35" s="59" t="inlineStr">
+      <c r="M35" s="79" t="inlineStr">
         <is>
           <t>R2 candidate (S6) ⚠ prioritaire</t>
         </is>
       </c>
-      <c r="N35" s="59" t="inlineStr">
+      <c r="N35" s="79" t="inlineStr">
         <is>
           <t>Corrige le moment de décrochage n°1 identifié sur le customer journey de Léa (étape 3).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="79.5" customHeight="1" s="41">
-      <c r="A36" s="58" t="inlineStr">
+      <c r="A36" s="76" t="inlineStr">
         <is>
           <t>US-24</t>
         </is>
       </c>
-      <c r="B36" s="59" t="inlineStr">
+      <c r="B36" s="79" t="inlineStr">
         <is>
           <t>EP-09</t>
         </is>
       </c>
-      <c r="C36" s="59" t="inlineStr">
+      <c r="C36" s="79" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux consulter mon historique sans connexion, afin de réviser dans les transports.</t>
         </is>
       </c>
-      <c r="D36" s="59" t="inlineStr">
+      <c r="D36" s="79" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -6318,67 +6318,67 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F36" s="59" t="n">
+      <c r="F36" s="79" t="n">
         <v>8</v>
       </c>
-      <c r="G36" s="59" t="inlineStr">
+      <c r="G36" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : cache local (IndexedDB/service worker) de l'historique des 10 derniers quizz]</t>
         </is>
       </c>
-      <c r="H36" s="59" t="inlineStr">
+      <c r="H36" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I36" s="59" t="inlineStr">
+      <c r="I36" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J36" s="59" t="inlineStr">
+      <c r="J36" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K36" s="59" t="inlineStr">
+      <c r="K36" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L36" s="59" t="inlineStr">
+      <c r="L36" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M36" s="59" t="inlineStr">
+      <c r="M36" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N36" s="59" t="inlineStr">
+      <c r="N36" s="79" t="inlineStr">
         <is>
           <t>8 SP : nécessite une stratégie de cache/synchronisation, pas un simple CRUD.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="79.5" customHeight="1" s="41">
-      <c r="A37" s="58" t="inlineStr">
+      <c r="A37" s="76" t="inlineStr">
         <is>
           <t>US-25</t>
         </is>
       </c>
-      <c r="B37" s="59" t="inlineStr">
+      <c r="B37" s="79" t="inlineStr">
         <is>
           <t>EP-10</t>
         </is>
       </c>
-      <c r="C37" s="59" t="inlineStr">
+      <c r="C37" s="79" t="inlineStr">
         <is>
           <t>En tant qu'étudiant·e, je veux partager un quiz avec mes amies de promo, afin qu'on révise ensemble.</t>
         </is>
       </c>
-      <c r="D37" s="59" t="inlineStr">
+      <c r="D37" s="79" t="inlineStr">
         <is>
           <t>Étudiant·e</t>
         </is>
@@ -6388,63 +6388,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F37" s="59" t="n">
+      <c r="F37" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="G37" s="59" t="inlineStr">
+      <c r="G37" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : lien de partage généré, quiz accessible en lecture par le destinataire]</t>
         </is>
       </c>
-      <c r="H37" s="59" t="inlineStr">
+      <c r="H37" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I37" s="59" t="inlineStr">
+      <c r="I37" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J37" s="59" t="inlineStr">
+      <c r="J37" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K37" s="59" t="inlineStr">
+      <c r="K37" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L37" s="59" t="inlineStr">
+      <c r="L37" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M37" s="59" t="inlineStr">
+      <c r="M37" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N37" s="59" t="n"/>
+      <c r="N37" s="79" t="n"/>
     </row>
     <row r="38" ht="79.5" customHeight="1" s="41">
-      <c r="A38" s="58" t="inlineStr">
+      <c r="A38" s="76" t="inlineStr">
         <is>
           <t>US-26</t>
         </is>
       </c>
-      <c r="B38" s="59" t="inlineStr">
+      <c r="B38" s="79" t="inlineStr">
         <is>
           <t>EP-01</t>
         </is>
       </c>
-      <c r="C38" s="59" t="inlineStr">
+      <c r="C38" s="79" t="inlineStr">
         <is>
           <t>En tant qu'enseignante, je veux créer mon compte immédiatement sans validation manuelle, afin de tester l'outil sans délai.</t>
         </is>
       </c>
-      <c r="D38" s="59" t="inlineStr">
+      <c r="D38" s="79" t="inlineStr">
         <is>
           <t>Enseignant·e</t>
         </is>
@@ -6454,67 +6454,67 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F38" s="59" t="n">
+      <c r="F38" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="G38" s="59" t="inlineStr">
+      <c r="G38" s="79" t="inlineStr">
         <is>
           <t>G: visiteur sur /signup-enseignant W: soumet email établissement + mdp T: compte enseignant créé immédiatement, aucune validation manuelle requise</t>
         </is>
       </c>
-      <c r="H38" s="59" t="inlineStr">
+      <c r="H38" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I38" s="59" t="inlineStr">
+      <c r="I38" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J38" s="59" t="inlineStr">
+      <c r="J38" s="79" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="K38" s="59" t="inlineStr">
+      <c r="K38" s="79" t="inlineStr">
         <is>
           <t>Todo</t>
         </is>
       </c>
-      <c r="L38" s="59" t="inlineStr">
+      <c r="L38" s="79" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="M38" s="59" t="inlineStr">
+      <c r="M38" s="79" t="inlineStr">
         <is>
           <t>R2 candidate (S6) ⚠ prioritaire</t>
         </is>
       </c>
-      <c r="N38" s="59" t="inlineStr">
+      <c r="N38" s="79" t="inlineStr">
         <is>
           <t>Corrige le moment de décrochage n°1 identifié sur le customer journey de Mme Lefèvre (étape 2).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="79.5" customHeight="1" s="41">
-      <c r="A39" s="58" t="inlineStr">
+      <c r="A39" s="76" t="inlineStr">
         <is>
           <t>US-27</t>
         </is>
       </c>
-      <c r="B39" s="59" t="inlineStr">
+      <c r="B39" s="79" t="inlineStr">
         <is>
           <t>EP-08</t>
         </is>
       </c>
-      <c r="C39" s="59" t="inlineStr">
+      <c r="C39" s="79" t="inlineStr">
         <is>
           <t>En tant qu'enseignante, je veux prévisualiser les questions avant de les publier, afin de vérifier leur pertinence.</t>
         </is>
       </c>
-      <c r="D39" s="59" t="inlineStr">
+      <c r="D39" s="79" t="inlineStr">
         <is>
           <t>Enseignant·e</t>
         </is>
@@ -6524,63 +6524,63 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F39" s="59" t="n">
+      <c r="F39" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="G39" s="59" t="inlineStr">
+      <c r="G39" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : écran de preview des 10 QCM avant le bouton 'Publier']</t>
         </is>
       </c>
-      <c r="H39" s="59" t="inlineStr">
+      <c r="H39" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I39" s="59" t="inlineStr">
+      <c r="I39" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J39" s="59" t="inlineStr">
+      <c r="J39" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K39" s="59" t="inlineStr">
+      <c r="K39" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L39" s="59" t="inlineStr">
+      <c r="L39" s="79" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="M39" s="59" t="inlineStr">
+      <c r="M39" s="79" t="inlineStr">
         <is>
           <t>Plus tard / stretch S7</t>
         </is>
       </c>
-      <c r="N39" s="59" t="n"/>
+      <c r="N39" s="79" t="n"/>
     </row>
     <row r="40" ht="79.5" customHeight="1" s="41">
-      <c r="A40" s="58" t="inlineStr">
+      <c r="A40" s="76" t="inlineStr">
         <is>
           <t>US-28</t>
         </is>
       </c>
-      <c r="B40" s="59" t="inlineStr">
+      <c r="B40" s="79" t="inlineStr">
         <is>
           <t>EP-06</t>
         </is>
       </c>
-      <c r="C40" s="59" t="inlineStr">
+      <c r="C40" s="79" t="inlineStr">
         <is>
           <t>En tant que directeur, je veux télécharger une fiche RGPD pré-rédigée, afin de la transmettre vite à mon DPO.</t>
         </is>
       </c>
-      <c r="D40" s="59" t="inlineStr">
+      <c r="D40" s="79" t="inlineStr">
         <is>
           <t>Établissement</t>
         </is>
@@ -6590,67 +6590,67 @@
           <t>SHOULD</t>
         </is>
       </c>
-      <c r="F40" s="59" t="n">
+      <c r="F40" s="79" t="n">
         <v>1</v>
       </c>
-      <c r="G40" s="59" t="inlineStr">
+      <c r="G40" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : bouton de téléchargement d'un PDF de 2 pages, contenu validé juridiquement]</t>
         </is>
       </c>
-      <c r="H40" s="59" t="inlineStr">
+      <c r="H40" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I40" s="59" t="inlineStr">
+      <c r="I40" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J40" s="59" t="inlineStr">
+      <c r="J40" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K40" s="59" t="inlineStr">
+      <c r="K40" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L40" s="59" t="inlineStr">
+      <c r="L40" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M40" s="59" t="inlineStr">
+      <c r="M40" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N40" s="59" t="inlineStr">
+      <c r="N40" s="79" t="inlineStr">
         <is>
           <t>Surtout un travail de contenu/juridique, peu de code.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="79.5" customHeight="1" s="41">
-      <c r="A41" s="58" t="inlineStr">
+      <c r="A41" s="76" t="inlineStr">
         <is>
           <t>US-29</t>
         </is>
       </c>
-      <c r="B41" s="59" t="inlineStr">
+      <c r="B41" s="79" t="inlineStr">
         <is>
           <t>EP-06</t>
         </is>
       </c>
-      <c r="C41" s="59" t="inlineStr">
+      <c r="C41" s="79" t="inlineStr">
         <is>
           <t>En tant que DPO, je veux une check-list RGPD pré-validée juridiquement, afin de valider les CGV rapidement.</t>
         </is>
       </c>
-      <c r="D41" s="59" t="inlineStr">
+      <c r="D41" s="79" t="inlineStr">
         <is>
           <t>Établissement</t>
         </is>
@@ -6660,63 +6660,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F41" s="59" t="n">
+      <c r="F41" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="G41" s="59" t="inlineStr">
+      <c r="G41" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : check-list interactive de 10 points, exportable en PDF]</t>
         </is>
       </c>
-      <c r="H41" s="59" t="inlineStr">
+      <c r="H41" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I41" s="59" t="inlineStr">
+      <c r="I41" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J41" s="59" t="inlineStr">
+      <c r="J41" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K41" s="59" t="inlineStr">
+      <c r="K41" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L41" s="59" t="inlineStr">
+      <c r="L41" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M41" s="59" t="inlineStr">
+      <c r="M41" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N41" s="59" t="n"/>
+      <c r="N41" s="79" t="n"/>
     </row>
     <row r="42" ht="79.5" customHeight="1" s="41">
-      <c r="A42" s="58" t="inlineStr">
+      <c r="A42" s="76" t="inlineStr">
         <is>
           <t>US-30</t>
         </is>
       </c>
-      <c r="B42" s="59" t="inlineStr">
+      <c r="B42" s="79" t="inlineStr">
         <is>
           <t>EP-11</t>
         </is>
       </c>
-      <c r="C42" s="59" t="inlineStr">
+      <c r="C42" s="79" t="inlineStr">
         <is>
           <t>En tant que directeur, je veux un kit de déploiement accessible depuis l'app, afin de garantir une adoption réussie.</t>
         </is>
       </c>
-      <c r="D42" s="59" t="inlineStr">
+      <c r="D42" s="79" t="inlineStr">
         <is>
           <t>Établissement</t>
         </is>
@@ -6726,63 +6726,63 @@
           <t>COULD</t>
         </is>
       </c>
-      <c r="F42" s="59" t="n">
+      <c r="F42" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="G42" s="59" t="inlineStr">
+      <c r="G42" s="79" t="inlineStr">
         <is>
           <t>[1 critère type : page ressources avec guides PDF + vidéos d'onboarding par rôle]</t>
         </is>
       </c>
-      <c r="H42" s="59" t="inlineStr">
+      <c r="H42" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I42" s="59" t="inlineStr">
+      <c r="I42" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J42" s="59" t="inlineStr">
+      <c r="J42" s="79" t="inlineStr">
         <is>
           <t>Backlog R3+</t>
         </is>
       </c>
-      <c r="K42" s="59" t="inlineStr">
+      <c r="K42" s="79" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="L42" s="59" t="inlineStr">
+      <c r="L42" s="79" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="M42" s="59" t="inlineStr">
+      <c r="M42" s="79" t="inlineStr">
         <is>
           <t>Plus tard (R3+)</t>
         </is>
       </c>
-      <c r="N42" s="59" t="n"/>
+      <c r="N42" s="79" t="n"/>
     </row>
     <row r="43" ht="79.5" customHeight="1" s="41">
-      <c r="A43" s="58" t="inlineStr">
+      <c r="A43" s="76" t="inlineStr">
         <is>
           <t>US-31</t>
         </is>
       </c>
-      <c r="B43" s="59" t="inlineStr">
+      <c r="B43" s="79" t="inlineStr">
         <is>
           <t>EP-06</t>
         </is>
       </c>
-      <c r="C43" s="59" t="inlineStr">
+      <c r="C43" s="79" t="inlineStr">
         <is>
           <t>En tant que directeur, je veux comparer mon adoption à la moyenne anonymisée d'autres écoles, afin de justifier le renouvellement.</t>
         </is>
       </c>
-      <c r="D43" s="59" t="inlineStr">
+      <c r="D43" s="79" t="inlineStr">
         <is>
           <t>Établissement</t>
         </is>
@@ -6792,45 +6792,45 @@
           <t>WON'T</t>
         </is>
       </c>
-      <c r="F43" s="59" t="n">
+      <c r="F43" s="79" t="n">
         <v>13</v>
       </c>
-      <c r="G43" s="59" t="inlineStr">
+      <c r="G43" s="79" t="inlineStr">
         <is>
           <t>Nécessite une base installée multi-établissements pour être pertinent. Reporté.</t>
         </is>
       </c>
-      <c r="H43" s="59" t="inlineStr">
+      <c r="H43" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="I43" s="59" t="inlineStr">
+      <c r="I43" s="79" t="inlineStr">
         <is>
           <t>□</t>
         </is>
       </c>
-      <c r="J43" s="59" t="inlineStr">
+      <c r="J43" s="79" t="inlineStr">
         <is>
           <t>n.c.</t>
         </is>
       </c>
-      <c r="K43" s="59" t="inlineStr">
+      <c r="K43" s="79" t="inlineStr">
         <is>
           <t>Won't</t>
         </is>
       </c>
-      <c r="L43" s="59" t="inlineStr">
+      <c r="L43" s="79" t="inlineStr">
         <is>
           <t>★★</t>
         </is>
       </c>
-      <c r="M43" s="59" t="inlineStr">
+      <c r="M43" s="79" t="inlineStr">
         <is>
           <t>Hors scope (WON'T)</t>
         </is>
       </c>
-      <c r="N43" s="59" t="inlineStr">
+      <c r="N43" s="79" t="inlineStr">
         <is>
           <t>13 SP = seuil de redécoupage. Dépend en plus d'un volume de clients qu'on n'a pas encore : à reporter en Release 3+, pas à découper maintenant.</t>
         </is>
@@ -6889,7 +6889,7 @@
       </c>
       <c r="K44" s="77" t="inlineStr">
         <is>
-          <t>Livré (MVP)</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="L44" s="79" t="inlineStr">
@@ -6904,7 +6904,7 @@
       </c>
       <c r="N44" s="79" t="inlineStr">
         <is>
-          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM, OWASP LLM-01). Responsable : Azeddine AMARI (TSEC-01). Voir docs/J3/backlog_sprint2.md.</t>
+          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM, OWASP LLM-01). Responsable : Azeddine AMARI (TSEC-01). Voir docs/J3/backlog_sprint2.md. Audit code 01/07 : séparation system/user confirmée pour OpenAI-compatible et Anthropic ; manquante pour Ollama. System prompt présent mais sans consignes anti-injection explicites robustes (T-SEC-01).</t>
         </is>
       </c>
     </row>
@@ -6961,7 +6961,7 @@
       </c>
       <c r="K45" s="77" t="inlineStr">
         <is>
-          <t>Livré (MVP)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L45" s="79" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="N45" s="79" t="inlineStr">
         <is>
-          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM). Responsable : Redouane ID SOUGOU (TSEC-02).</t>
+          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM). Responsable : Redouane ID SOUGOU (TSEC-02). Audit code 01/07 : validation stricte confirmée (10 questions, 4 options, correct_index 0-3, exception LLMError) dans llm/services/quiz_prompt.py (T-SEC-02).</t>
         </is>
       </c>
     </row>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="K46" s="77" t="inlineStr">
         <is>
-          <t>Livré (MVP)</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="L46" s="79" t="inlineStr">
@@ -7048,7 +7048,7 @@
       </c>
       <c r="N46" s="79" t="inlineStr">
         <is>
-          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM). Responsable : Romain LEFEVRE (TSEC-03).</t>
+          <t>Nouvelle US issue de la perturbation J3 (sécurité LLM). Responsable : Romain LEFEVRE (TSEC-03). Audit code 01/07 : aucun test adversarial (prompt injection / XSS) trouvé dans le repo (T-SEC-03).</t>
         </is>
       </c>
     </row>
@@ -7068,7 +7068,7 @@
       </c>
       <c r="G47" s="81" t="inlineStr">
         <is>
-          <t>37 stories · 25 SP verrouillés en R1 (MVP) · 14 SP livrés J3 (5 RGPD US-RGPD-01/02 + 8 sécurité LLM US-SEC-01/02/03) · 14 SP retenus en R2 candidate (US-23, US-26, US-T1) · reste en Plus tard / Hors scope</t>
+          <t>37 stories · 25 SP verrouillés en R1 (MVP) · 14 SP engagés J3 (statuts en cours de vérification) (5 RGPD US-RGPD-01/02 + 8 sécurité LLM US-SEC-01/02/03) · 14 SP retenus en R2 candidate (US-23, US-26, US-T1) · reste en Plus tard / Hors scope</t>
         </is>
       </c>
       <c r="H47" s="81" t="n"/>

</xml_diff>